<commit_message>
WIP checkpoint: capture v2 branch baseline.
Freeze current scoring, docs, and backtest artifacts on a dedicated v2 branch for review and follow-up iteration.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backtests/datasets/CoCo_examples.xlsx
+++ b/backtests/datasets/CoCo_examples.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onedrive-global.kpmg.com/personal/weiliu3_kpmg_com_sg/Documents/Documents/Projects/Project X/CoCo AI Agent/Design/CoCos examples/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onedrive-global.kpmg.com/personal/weiliu3_kpmg_com_sg/Documents/Documents/Projects/Project X/CoCo AI Agent/CoCo_AI/backtests/datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="11_F25DC773A252ABDACC10482A91DA41D85ADE58F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BDB02AB-6AA0-458E-919F-2B1C58279036}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="11_F25DC773A252ABDACC10482A91DA41D85ADE58F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7F84E9B-6CCC-4DD2-9ED7-A6F4612EB38E}"/>
   <bookViews>
     <workbookView xWindow="14580" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -617,7 +617,7 @@
         <v>Vuzix Corporation designs, manufactures, and markets artificial intelligence (AI)-powered smart glasses, waveguides, and augmented reality (AR) technologies in North America, Europe, the Asia Pacific, and internationally. The company offers smart glasses that include M Series, Vuzix Blade, Vuzix Shield, and Vuzix Ultralite Z100; Mobilium logistics mobility software solution; waveguide optics; and display engines. It provides engineering services and original design manufacturers (ODM)/original equipment manufacturers (OEM) component solutions. It also offers head-mounted smart display and wearable computing devices. The company sells its products through direct sales, value-added resellers, distributors, ODM and OEM partnerships, and online stores, as well as various Vuzix operated web stores in the United States, Europe, and Japan. It serves the enterprise, medical, defense, security, and consumer markets. The company was formerly known as Icuiti Corporation and changed its name to Vuzix Corporation in September 2007. Vuzix Corporation was incorporated in 1997 and is headquartered in West Henrietta, New York.</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -626,7 +626,7 @@
         <v>Cosonic Intelligent Technologies Co., Ltd. engages in the design, development, manufacture, and sale of electroacoustic and smart wearable products in China and internationally. The company offers electro-acoustic products, such as TWS earphones, bone conduction earphones, smart speakers, etc.; smart wearable products, including smart watches, smart glasses, etc., as well as audio glasses, bone conduction glasses, VR/AR, etc. It also offers full-voice AI translation earphones, wireless heart rate monitoring earphones, voice-interactive AI speaker, neckband Bluetooth smart headphones, portable bluetooth speaker, and smart charger. Cosonic Intelligent Technologies Co., Ltd. was founded in 2013 and is based in Dongguan, China.</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -635,7 +635,7 @@
         <v>Jorjin Technologies Inc. engages in the research, development, design, manufacture, and trading of electronic components and its products in Taiwan, China, the United States, Europe, and internationally. It offers ultra-light AR glasses and industrial AR solution. The company was incorporated in 1997 and is based in New Taipei City, Taiwan.</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -644,7 +644,7 @@
         <v>XMReality AB (publ) provides remote visual assistance solution in Sweden, European Union, North America, and internationally. The company offers Remote Guidance, a remote support software and video calling solution built for service, support, inspection, and training; and provides Pointpad, a hardware add-on that transforms desktop into a remote support station; and AR smart glasses. It serves manufacturing, heating and cooling, renewable energy, and housing and facility management industries. The company was incorporated in 2007 and is based in Linköping, Sweden.</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -653,7 +653,7 @@
         <v>Garmin Ltd. designs, develops, manufactures, markets, and distributes a diverse range of GPS-enabled products and navigation, communications, sensor-based, and information products and services worldwide. It offers running; cycling products; smartwatch devices; scales and monitors; and sports timing and performance analysis; Garmin Connect and Garmin Connect Mobile, which are web and mobile platforms where users can track and analyze their fitness, activities and workouts, and wellness data; and Connect IQ, which enables third parties to create applications that run on Garmin devices. It also provides adventure watches; outdoor handhelds and satellite communicators; golf devices; consumer automotive; dog devices; InReach and Gramin response; and dive devices. In addition, it designs, manufactures, and markets various aircraft avionics solutions, including integrated flight decks, electronic flight displays and instrumentation, navigation and communication products, automatic flight control systems and safety-enhancing technologies, audio control systems, engine indication systems, traffic awareness and avoidance solutions, ADS-B and transponders, weather information and avoidance solutions, datalink and connectivity solutions, and portable GPS navigators and wearables, as well as service products to the aviation market. Further, it offers chartplotters and multi-function displays, cartography, fishfinders, sonar, autopilot systems, radars, compliant instrument displays and sensors, VHF communication radios, handhelds and wearable devices, sailing, audio, digital switching, trolling motors, and lighting; and domain controllers and infotainment units, as well as software, map database, camera, wearable, and automotive solutions. The company sells its products through independent retailers, dealers, distributors, installation and repair shops, OEM, and online webshop. Garmin Ltd. was founded in 1989 and is based in Schaffhausen, Switzerland.</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -662,7 +662,7 @@
         <v>ARway Corporation engages in developing and operating of intellectual property applications in Canada. The company offers ARway, a mobile app no code Metaverse creation tool with self-generating AR mapping solutions for consumers and brands. It also provides ARwayKit SDK, which offers resources to build new apps; ARway creator portal, a suite of tools for floorplan configuration, AR navigation creation, and detailed analytics; and smart glasses operated using artificial intelligence. Its products are used in various industries, including stadiums and concert venues, events and tradeshows, retail, museums and galleries, hospitality, real estate, universities, hospitals, and other sectors. ARway Corporation was incorporated in 2022 and is headquartered in Toronto, Canada.</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -671,7 +671,7 @@
         <v>Wearable Devices Ltd. engages in the development of a non-invasive neural input interface for controlling digital devices using subtle touchless finger movements. The company offers Mudra development kits that enable users to control digital devices, including consumer electronics, smart watches, smartphones, augmented reality glasses, virtual reality headsets, televisions, personal and laptop computers, drones, robots, and others through finger movements and hand gestures; and SNC sensor module, an operating system software and algorithm software package. It also provides Mudra Band, a neural input wristband, which allows users to control Apple ecosystem devices, including iPhone, Mac computer, Apple TV, iPad, and Apple Vision Pro using subtle touchless finger movements and gestures and Mudra Link, a universal personalized gesture control neural band that allows users to control any Bluetooth compatible device regardless of the operating system. The company serves consumer electronics companies, consumer electronics brands, industrial manufacturing companies, IT and software solutions providers, software development studios, and academic institutions. The company was incorporated in 2014 and is headquartered in Yokneam Illit, Israel.</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
@@ -710,7 +710,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -719,7 +719,7 @@
         <v>Baoxiniao Holding Co., Ltd. engages in the research and development, production, and sale of branded men and women clothing products in China. Its products include suits, trousers, shirts, jackets, sheep sweaters, POLO shirts, down jackets, quick-drying clothes, casual pants, leather shoes, and leather goods. The company sells its products through retail market, e-commerce, live broadcasting, online and offline channels under the SAINT ANGELO, Baoxiniao, HAZZYS, Baoniao, SOLOSALI, Camicissima, Lafuma, Dombolini, HENRY GRANT, elitebasic, BONO, and Ashwell brand names. In addition, it is involved in industrial investment. The company was formerly known as Zhejiang Baoxiniao Garment Co., Ltd and changed its name to Baoxiniao Holding Co., Ltd. in 2017. Baoxiniao Holding Co., Ltd. was founded in 2001 and is headquartered in Wenzhou, China.</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" ht="116" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>15</v>
       </c>
@@ -728,7 +728,7 @@
         <v>Fujian Septwolves Industry Co., Ltd. engages in the research and development, design, manufacturing, and sales of clothing and apparel products and raw material in China and internationally. The company offers men’s shirts, suits, trousers, jackets, sweaters, underwear, briefs, socks, and other knitting products under the Seven Wolves brand name. It is involved in embroidery and printing processing, property management, and house rental operations; sales training and consulting activities; interior decoration business; general merchandise; department store sales; and foreign trade and venture capital. In addition, the company provides building materials; computer software and hardware services; and hardware and electrical appliances. It sells its products through franchise stores and online. The company was formerly known as Fujian Septwolves Garment Industry Co., Ltd. and changed its name to Fujian Septwolves Industry Co., Ltd. in July 2001. The company was founded in 1989 and is based in Jinjiang, China.</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -737,7 +737,7 @@
         <v>Cedar Development Co.,Ltd. provides supply chain management services in China. The company offers supply chain services for the production and sales of coal, coke, aluminum, oil products, and steel products through Cedar Smart Chain platform. It also engages in the development and operation of cultural tourism business. The company was formerly known as Sinoer Men's Wear Co., Ltd. and changed its name to Cedar Development Co., Ltd. in August 2021. The company was founded in 2003 and is based in Guangzhou, China.</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -755,7 +755,7 @@
         <v>Pearl Global Industries Limited, together with its subsidiaries, manufactures and sells readymade garments in India and internationally. The company offers tops, shirts, long shirts, dresses, sleepwear, hoodies, leggings, skirts, sweaters, t-shirts, joggers for women; shirts, polo t-shirts, sleepwear, pyjamas, and hoodies for men; t-shirts, shirts, and two-piece sets for boys; tops, t-shirts, skirts, dresses, rompers, and tank tops for girls; and rompers for toddlers. It also provides activewear, athleisure, children’s wear, workwear, and denim apparels. In addition, the company is involved in the trading of garments online; and skill development business, as well as provides end-to-end supply chain solutions. It provides its products through retailers. The company was formerly known as House of Pearl Fashions Limited. Pearl Global Industries Limited was incorporated in 1987 and is based in Gurugram, India.</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
@@ -764,7 +764,7 @@
         <v>Tainan Enterprises Co., Ltd., together with its subsidiaries, engages in the manufacturing, retail, and export of woven and knitted garments. It offers ready-to-wear, active wear, sleep wears, uniforms, and denim products, as well as accessories; and professional investment services. The company serves clients in the United States, Canada, Japan, China, Taiwan, Cambodia, Vietnam, Indonesia, and internationally. Tainan Enterprises Co., Ltd. was incorporated in 1961 and is based in Taipei, Taiwan.</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>20</v>
       </c>
@@ -773,7 +773,7 @@
         <v>Daidoh Limited manufactures and sells ready-made men's and women’s clothing and accessories in Japan. The company offers custom made clothing products, knitted yarns, worsted fabrics, apparel, etc. It also provides OEM, as well as import and export services. In addition, the company manufactures, sells, and retails yarns, fibrous materials for apparel, and apparel. Further, it sells its products under the NEWYORKER, Brooks Brothers, and House Tartan brands. Further, the company is involved in the leasing of real-estate properties, such as shopping center stores, office buildings, and hotel facilities. The company was founded in 1879 and is headquartered in Tokyo, Japan.</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>21</v>
       </c>
@@ -782,7 +782,7 @@
         <v>Shanghai Metersbonwe Fashion and Accessories Co., Ltd., together with its subsidiaries, engages in the design, promotion, and sale of apparel products in the People’s Republic of China. The company operates through the Wholesale Business, Retail Business, and Other Business segments. It is involved in the wholesale and retail sale of adults’ and children’s clothing products under the Metersbonwe, ME&amp;CITY, ME&amp;CITYKIDS, and MooMoo brand names through offline store channels and internet e-commerce platforms. The company was founded in 1995 and is headquartered in Shanghai, China.</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
@@ -791,7 +791,7 @@
         <v>ONTIDE Corp. manufactures and sells textile products in Mexico, Indonesia, Vietnam, Bangladesh, and the Philippines. It also offers active sportswear, such as athleisure, teamwear, and golf wear; lifestyle wear; and workwear. The company also exports its products. The company was formerly known as Kukdong Corporation and changed its name to ONTIDE Corp. in October 2024. ONTIDE Corp. was founded in 1967 and is headquartered in Seoul, South Korea.</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" ht="203" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>23</v>
       </c>
@@ -800,7 +800,7 @@
         <v>Greatime International Holdings Limited, an investment holding company, manufactures and sells knitted fabrics and innerwear products for infants and adults in the People’s Republic of China. The company operates through Innerwear Products; Knitted Fabrics; and Space Measurement Services, Industrial Drones, and Measurement Robots segments. It is involved in the provision of functional and customized fabrics for lingerie and apparel brands; and a range of innerwear for men, women, toddlers, and infants, including T-shirts, vests, long-sleeves pullovers, men’s briefs and boxer briefs, women’s panties, long johns, and toddlers’ and infants’ body suits and bibs. The company also manufactures and trades in garments; and offers fabric weaving, knitting, printing, and dyeing services. In addition, it engages in the provision of high-precision space measurement and modelling services; geographic spatial data measurement services; internal and external industry software development; and CIM underlying platform and system construction; as well as research and development, production, sale, and technical assistance of industrial drones and 3D high-precision laser radar measuring robots. The company primarily sells its products to the sourcing agents, wholesalers, and brand owners. It also has operations in Japan, Taiwan, Italy, Africa, Hong Kong, the Netherlands, the United States, Germany, Myanmar, Southeast Asia, and Norway. The company was formerly known as Grand Concord International Holdings Limited and changed its name to Greatime International Holdings Limited in June 2017. Greatime International Holdings Limited was founded in 2000 and is headquartered in Admiralty, Hong Kong. Greatime International Holdings Limited is a subsidiary of Junfun Investment Limited.</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>24</v>
       </c>
@@ -809,7 +809,7 @@
         <v>Hla Group Corp., Ltd. manufactures and sells menswear, womenswear, kids, professional, and home furnishing products in China and internationally. The company offers T-shirts, trousers, shirts, coats, windbreakers, shoes, suits, jackets, down jackets, sweaters, knitwear, home furnishings, accessories, luggage, glasses, vests, skirts, sleeping bag, baby carriage, crib, and other products under the HLA; HLA JEANS; OVV; YeeHoO; and HLAF2C brands. The company was formerly known as HLA CORP., Ltd. and changed its name to Hla Group Corp., Ltd. in March 2021. Hla Group Corp., Ltd. was founded in 1997 and is based in Jiangyin, China.</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" ht="116" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>25</v>
       </c>

</xml_diff>